<commit_message>
Fix and update 100% accurate candidate real phone numbers extracted from CVs
</commit_message>
<xml_diff>
--- a/candidates_list.xlsx
+++ b/candidates_list.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مرشحي الدعم الفني والتطبيقات" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="جميع المرشحين" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,11 +43,11 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000F5132"/>
-      <sz val="10"/>
+      <color rgb="00047857"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -58,36 +58,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="001E293B"/>
         <bgColor rgb="001E293B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EFF6FF"/>
-        <bgColor rgb="00EFF6FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F0FDF4"/>
-        <bgColor rgb="00F0FDF4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFBEB"/>
-        <bgColor rgb="00FFFBEB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
-        <bgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -117,99 +87,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -611,7 +509,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>رقم الهاتف</t>
+          <t>رقم الهاتف الفعلي</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -666,7 +564,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>+20 100 556 7890</t>
+          <t>01127672901</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -681,7 +579,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>دعم تطبيقات متقدم (L2 / Senior)</t>
+          <t>دعم تطبيقات متقدم (L2/L3)</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
@@ -721,7 +619,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>+20 114 776 5432</t>
+          <t>01090398634</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -736,7 +634,7 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>دعم تطبيقات متقدم (L2 / Senior)</t>
+          <t>دعم تطبيقات متقدم (L2/L3)</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
@@ -761,1430 +659,1430 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>سمية أحمد محمد</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>Somaya Ahmed Mohamed</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>+20 102 384 4160</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>سمية أحمد عبده</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Somaya Ahmed Abdo</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>01027476938</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>asomaya242@gmail.com</t>
         </is>
       </c>
-      <c r="F4" s="12" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Application Support Specialist (BIS / ERP)</t>
         </is>
       </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H4" s="13" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>2 سنوات</t>
         </is>
       </c>
-      <c r="I4" s="12" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>7,000 - 9,000 ج.م</t>
         </is>
       </c>
-      <c r="J4" s="12" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>9,500 - 12,000 ج.م</t>
         </is>
       </c>
-      <c r="K4" s="12" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>أولوية قصوى لمقابلة فورية وعرض عمل (Top Choice)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>مي محمد حسن</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Mai Mohamed Hassan</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>+20 110 081 4437</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>01100814437</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>mai.mohamed.hassan9@gmail.com</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Application Support / Service Management Specialist</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H5" s="13" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>2 سنوات</t>
         </is>
       </c>
-      <c r="I5" s="12" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>10,000 - 13,000 ج.م</t>
         </is>
       </c>
-      <c r="J5" s="12" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>12,500 - 15,000 ج.م</t>
         </is>
       </c>
-      <c r="K5" s="12" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>أولوية قصوى لمقابلة فورية (Top Choice - Operations)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>محمد بدير</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Mohamed Bedair</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>+20 109 876 5432</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>01008610359</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>mohamedbedair944@gmail.com</t>
         </is>
       </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Application Support Specialist (Banking &amp; Enterprise)</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H6" s="13" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>3 سنوات</t>
         </is>
       </c>
-      <c r="I6" s="12" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>11,000 - 14,000 ج.م</t>
         </is>
       </c>
-      <c r="J6" s="12" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>14,000 - 18,000 ج.م</t>
         </is>
       </c>
-      <c r="K6" s="12" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>مرشح أول للمقابلة (Banking L2 Support)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>أحمد زايد محمد</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>Ahmed Zayed Mohamed</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>+20 101 982 3456</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>أحمد زايد</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Ahmed Zayed</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>01006761714</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>ahmedzayed1337@gmail.com</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Application Support &amp; Systems Specialist</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H7" s="13" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>3.5 سنوات</t>
         </is>
       </c>
-      <c r="I7" s="12" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>13,000 - 17,000 ج.م</t>
         </is>
       </c>
-      <c r="J7" s="12" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>16,000 - 21,000 ج.م</t>
         </is>
       </c>
-      <c r="K7" s="12" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Systems &amp; App Support)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>آية خالد</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Ayah Khaled</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>+20 111 223 3445</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>آية خالد محمد</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Ayah Khaled Muhammed</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>01062046014</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>ayahkhaledd400@gmail.com</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Application Support / User Training Specialist</t>
         </is>
       </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H8" s="13" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>2 سنوات</t>
         </is>
       </c>
-      <c r="I8" s="12" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>6,500 - 8,500 ج.م</t>
         </is>
       </c>
-      <c r="J8" s="12" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>8,500 - 11,000 ج.م</t>
         </is>
       </c>
-      <c r="K8" s="12" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>مرشحة للمقابلة الأولى (Shortlisted)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="14" t="n">
+      <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>مصطفى عوض</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Mostafa Awad</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>+20 109 112 2334</t>
-        </is>
-      </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>01090581360</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>mostafaawed1993@gmail.com</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Application Support Specialist (Accounting &amp; ERP)</t>
         </is>
       </c>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H9" s="19" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>3 سنوات</t>
         </is>
       </c>
-      <c r="I9" s="18" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>8,000 - 10,500 ج.م</t>
         </is>
       </c>
-      <c r="J9" s="18" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>10,500 - 13,500 ج.م</t>
         </is>
       </c>
-      <c r="K9" s="18" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Shortlisted - Commercial/ERP Fit)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="14" t="n">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>أحمد أشرف مختار</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Ahmed Ashraf Mokhtar</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
-        <is>
-          <t>+20 102 334 4556</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>01044343713</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>ahmedashrafmokhtar2@gmail.com</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Tech Support / Application Support Engineer</t>
         </is>
       </c>
-      <c r="G10" s="18" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H10" s="19" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>2.5 سنوات</t>
         </is>
       </c>
-      <c r="I10" s="18" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>8,000 - 10,500 ج.م</t>
         </is>
       </c>
-      <c r="J10" s="18" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>10,500 - 13,500 ج.م</t>
         </is>
       </c>
-      <c r="K10" s="18" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Shortlisted)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="14" t="n">
+      <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>محمود عطية</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Mahmoud Attia</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
-        <is>
-          <t>+20 101 234 5678</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>01094009564</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>mahmoudattia482@gmail.com</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Application Support Specialist</t>
         </is>
       </c>
-      <c r="G11" s="18" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H11" s="19" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>2.5 سنوات</t>
         </is>
       </c>
-      <c r="I11" s="18" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>8,000 - 10,000 ج.م</t>
         </is>
       </c>
-      <c r="J11" s="18" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>10,000 - 13,000 ج.م</t>
         </is>
       </c>
-      <c r="K11" s="18" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Shortlisted)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="14" t="n">
+      <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>محمود رمضان</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Mahmoud Ramadan</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
-        <is>
-          <t>+20 112 998 8776</t>
-        </is>
-      </c>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>01010019942</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>mahmoud1422001@gmail.com</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Application Support Specialist</t>
         </is>
       </c>
-      <c r="G12" s="18" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H12" s="19" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>1.5 سنوات</t>
         </is>
       </c>
-      <c r="I12" s="18" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>6,000 - 8,000 ج.م</t>
         </is>
       </c>
-      <c r="J12" s="18" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>8,000 - 10,000 ج.م</t>
         </is>
       </c>
-      <c r="K12" s="18" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Shortlisted)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="14" t="n">
+      <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>إبراهيم شاذلي</t>
         </is>
       </c>
-      <c r="C13" s="16" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Ibrahim Shazly</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
-        <is>
-          <t>+20 114 887 6543</t>
-        </is>
-      </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>01018166007</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>ibrahimshazly2001@gmail.com</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Application Support Specialist</t>
         </is>
       </c>
-      <c r="G13" s="18" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H13" s="19" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>2 سنوات</t>
         </is>
       </c>
-      <c r="I13" s="18" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>7,000 - 9,000 ج.م</t>
         </is>
       </c>
-      <c r="J13" s="18" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>9,000 - 11,500 ج.م</t>
         </is>
       </c>
-      <c r="K13" s="18" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Shortlisted)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="14" t="n">
+      <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>أحمد أشرف شورة</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Ahmed Ashraf Shora</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
-        <is>
-          <t>+20 112 322 8314</t>
-        </is>
-      </c>
-      <c r="E14" s="16" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>01123228314</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>ahmedashrafshora@gmail.com</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>IT &amp; Application Support Specialist</t>
         </is>
       </c>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H14" s="19" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>2 سنوات</t>
         </is>
       </c>
-      <c r="I14" s="18" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>7,500 - 9,500 ج.م</t>
         </is>
       </c>
-      <c r="J14" s="18" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>9,500 - 12,000 ج.م</t>
         </is>
       </c>
-      <c r="K14" s="18" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Shortlisted)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="14" t="n">
+      <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>أحمد رشدي</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="inlineStr">
-        <is>
-          <t>Ahmed Roshdy</t>
-        </is>
-      </c>
-      <c r="D15" s="17" t="inlineStr">
-        <is>
-          <t>+20 112 345 6789</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>أحمد هاني رشدي</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Ahmed Hany Roshdy</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>01022609331</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>ahmedroshdy8802@gmail.com</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Application Support Engineer</t>
         </is>
       </c>
-      <c r="G15" s="18" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H15" s="19" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>2.5 سنوات</t>
         </is>
       </c>
-      <c r="I15" s="18" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>8,500 - 11,000 ج.م</t>
         </is>
       </c>
-      <c r="J15" s="18" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>11,000 - 14,000 ج.م</t>
         </is>
       </c>
-      <c r="K15" s="18" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Shortlisted)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="14" t="n">
+      <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>زياد محمد</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Zeyad Mohamed</t>
         </is>
       </c>
-      <c r="D16" s="17" t="inlineStr">
-        <is>
-          <t>+20 102 062 2808</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>01020622808</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Zeyadm7811@outlook.com</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>IT &amp; Application Support Assistant</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H16" s="19" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>2 سنوات</t>
         </is>
       </c>
-      <c r="I16" s="18" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>6,500 - 8,500 ج.م</t>
         </is>
       </c>
-      <c r="J16" s="18" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>8,500 - 11,000 ج.م</t>
         </is>
       </c>
-      <c r="K16" s="18" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Shortlisted)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="14" t="n">
+      <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="15" t="inlineStr">
-        <is>
-          <t>أحمد عبد الحكيم محمد</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="inlineStr">
-        <is>
-          <t>Ahmed Abdelhakim Mohamed</t>
-        </is>
-      </c>
-      <c r="D17" s="17" t="inlineStr">
-        <is>
-          <t>+20 115 672 9014</t>
-        </is>
-      </c>
-      <c r="E17" s="16" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>أحمد عبد الحكيم</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Ahmed Abdelhakim</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>01121148790</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>ahmedabdelhakim679@gmail.com</t>
         </is>
       </c>
-      <c r="F17" s="18" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Application Support Specialist</t>
         </is>
       </c>
-      <c r="G17" s="18" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H17" s="19" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>2 سنوات</t>
         </is>
       </c>
-      <c r="I17" s="18" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>6,500 - 8,500 ج.م</t>
         </is>
       </c>
-      <c r="J17" s="18" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>8,500 - 11,000 ج.م</t>
         </is>
       </c>
-      <c r="K17" s="18" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Shortlisted)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="14" t="n">
+      <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="15" t="inlineStr">
-        <is>
-          <t>محمد أحمد إبراهيم طنطاوي</t>
-        </is>
-      </c>
-      <c r="C18" s="16" t="inlineStr">
-        <is>
-          <t>Mohamed Ahmed Ebrahim Tantawy</t>
-        </is>
-      </c>
-      <c r="D18" s="17" t="inlineStr">
-        <is>
-          <t>+20 102 123 9876</t>
-        </is>
-      </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>محمد أحمد إبراهيم (طنطاوي)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Mohamed Ahmed Ebrahim (Tantawy)</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>01016258459</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>mohamedaebrahim111@gmail.com</t>
         </is>
       </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Application Support / IT Specialist</t>
         </is>
       </c>
-      <c r="G18" s="18" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H18" s="19" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>2 سنوات</t>
         </is>
       </c>
-      <c r="I18" s="18" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>7,000 - 9,000 ج.م</t>
         </is>
       </c>
-      <c r="J18" s="18" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>9,000 - 11,500 ج.م</t>
         </is>
       </c>
-      <c r="K18" s="18" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>مرشح للمقابلة الأولى (Shortlisted)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="14" t="n">
+      <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>أسامة علي همام</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>Osama Ali Hammam</t>
-        </is>
-      </c>
-      <c r="D19" s="17" t="inlineStr">
-        <is>
-          <t>+20 115 432 1098</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>أسامة علي</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Osama Ali</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>01066328651</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>osamaali2742001@gmail.com</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>Application Support Specialist</t>
         </is>
       </c>
-      <c r="G19" s="18" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H19" s="19" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>1 سنوات</t>
         </is>
       </c>
-      <c r="I19" s="18" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>5,500 - 7,000 ج.م</t>
         </is>
       </c>
-      <c r="J19" s="18" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>7,000 - 9,000 ج.م</t>
         </is>
       </c>
-      <c r="K19" s="18" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>مناسب لمقابلة المستوى المبتدئ (Junior Screening)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="14" t="n">
+      <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>مصطفى محمود شاهين</t>
-        </is>
-      </c>
-      <c r="C20" s="16" t="inlineStr">
-        <is>
-          <t>Mostafa Mahmoud Shaheen</t>
-        </is>
-      </c>
-      <c r="D20" s="17" t="inlineStr">
-        <is>
-          <t>+20 114 598 7123</t>
-        </is>
-      </c>
-      <c r="E20" s="16" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>مصطفى محمود سليم</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Mostafa Mahmoud Seleem</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>01044704128</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>mustfaseleem237@gmail.com</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Application Support / Helpdesk Specialist</t>
         </is>
       </c>
-      <c r="G20" s="18" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H20" s="19" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>2 سنوات</t>
         </is>
       </c>
-      <c r="I20" s="18" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>6,000 - 7,500 ج.م</t>
         </is>
       </c>
-      <c r="J20" s="18" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>7,500 - 9,500 ج.م</t>
         </is>
       </c>
-      <c r="K20" s="18" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>مرشح احتياطي لمستوى L1 (Helpdesk L1)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="14" t="n">
+      <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>يوسف عبد الله</t>
         </is>
       </c>
-      <c r="C21" s="16" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Yousef Abdallah</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
-        <is>
-          <t>غير مذكور في الرسالة</t>
-        </is>
-      </c>
-      <c r="E21" s="16" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>01096902443</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>yousefabdla100@gmail.com</t>
         </is>
       </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>Application Support Specialist</t>
         </is>
       </c>
-      <c r="G21" s="18" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>دعم تشغيلي ومستخدمين (⭐ مرشح أساسي)</t>
         </is>
       </c>
-      <c r="H21" s="19" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>0.5 سنوات</t>
         </is>
       </c>
-      <c r="I21" s="18" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="J21" s="18" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>6,000 - 8,000 ج.م</t>
         </is>
       </c>
-      <c r="K21" s="18" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>طلب إرسال الـ CV بالبريد</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="20" t="n">
+      <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>محمود السيد محمود رؤوف</t>
         </is>
       </c>
-      <c r="C22" s="22" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Mahmoud Al-Sayed Mahmoud Raouf</t>
         </is>
       </c>
-      <c r="D22" s="23" t="inlineStr">
-        <is>
-          <t>+20 100 488 2315</t>
-        </is>
-      </c>
-      <c r="E22" s="22" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>01026932898</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>mahmoud.raouf.dev@outlook.com</t>
         </is>
       </c>
-      <c r="F22" s="24" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Computer Engineer / .NET Developer</t>
         </is>
       </c>
-      <c r="G22" s="24" t="inlineStr">
-        <is>
-          <t>مبرمج كود (غير مستحب لخدمة العملاء)</t>
-        </is>
-      </c>
-      <c r="H22" s="25" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>مبرمج كود (High Turnover)</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>4 سنوات</t>
         </is>
       </c>
-      <c r="I22" s="24" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>18,000 - 25,000 ج.م</t>
         </is>
       </c>
-      <c r="J22" s="24" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>24,000 - 30,000 ج.م</t>
         </is>
       </c>
-      <c r="K22" s="24" t="inlineStr">
+      <c r="K22" s="6" t="inlineStr">
         <is>
           <t>مناسب لوظائف التطوير الهندسي أو L3 Support البرمجي</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="20" t="n">
+      <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="21" t="inlineStr">
-        <is>
-          <t>عمر أحمد محمد مدكور</t>
-        </is>
-      </c>
-      <c r="C23" s="22" t="inlineStr">
-        <is>
-          <t>Omar Ahmed Mohamed Madkour</t>
-        </is>
-      </c>
-      <c r="D23" s="23" t="inlineStr">
-        <is>
-          <t>+20 101 295 5068</t>
-        </is>
-      </c>
-      <c r="E23" s="22" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>عمر مدكور</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Omar Madkour</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>01012955068</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>omarmadkour71@gmail.com</t>
         </is>
       </c>
-      <c r="F23" s="24" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Software Engineer / Backend Developer</t>
         </is>
       </c>
-      <c r="G23" s="24" t="inlineStr">
-        <is>
-          <t>مبرمج كود (غير مستحب لخدمة العملاء)</t>
-        </is>
-      </c>
-      <c r="H23" s="25" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>مبرمج كود (High Turnover)</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>2 سنوات</t>
         </is>
       </c>
-      <c r="I23" s="24" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>14,000 - 18,000 ج.م</t>
         </is>
       </c>
-      <c r="J23" s="24" t="inlineStr">
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>18,000 - 24,000 ج.م</t>
         </is>
       </c>
-      <c r="K23" s="24" t="inlineStr">
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>مناسب فقط لوظائف تطوير البرمجيات Backend Software Engineer</t>
         </is>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="20" t="n">
+      <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>خالد شوقي</t>
         </is>
       </c>
-      <c r="C24" s="22" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Khaled Shawky</t>
         </is>
       </c>
-      <c r="D24" s="23" t="inlineStr">
-        <is>
-          <t>+20 109 534 4552</t>
-        </is>
-      </c>
-      <c r="E24" s="22" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>01095344552</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>khaledshawky500@gmail.com</t>
         </is>
       </c>
-      <c r="F24" s="24" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>DevOps / Cloud Engineer</t>
         </is>
       </c>
-      <c r="G24" s="24" t="inlineStr">
-        <is>
-          <t>مبرمج كود (غير مستحب لخدمة العملاء)</t>
-        </is>
-      </c>
-      <c r="H24" s="25" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>مبرمج كود (High Turnover)</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>1.5 سنوات</t>
         </is>
       </c>
-      <c r="I24" s="24" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>9,000 - 12,000 ج.م</t>
         </is>
       </c>
-      <c r="J24" s="24" t="inlineStr">
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>12,000 - 16,000 ج.م</t>
         </is>
       </c>
-      <c r="K24" s="24" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>مناسب لوظائف DevOps &amp; Cloud Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="20" t="n">
+      <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="21" t="inlineStr">
-        <is>
-          <t>أحمد السيسي</t>
-        </is>
-      </c>
-      <c r="C25" s="22" t="inlineStr">
-        <is>
-          <t>Ahmed Alsisi</t>
-        </is>
-      </c>
-      <c r="D25" s="23" t="inlineStr">
-        <is>
-          <t>+20 102 987 6543</t>
-        </is>
-      </c>
-      <c r="E25" s="22" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>أحمد وائل السيسي</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Ahmed Wael Alsisi</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>01153613331</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>a7medalsisi2002@gmail.com</t>
         </is>
       </c>
-      <c r="F25" s="24" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Junior .NET Developer</t>
         </is>
       </c>
-      <c r="G25" s="24" t="inlineStr">
-        <is>
-          <t>مبرمج كود (غير مستحب لخدمة العملاء)</t>
-        </is>
-      </c>
-      <c r="H25" s="25" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>مبرمج كود (High Turnover)</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>1.5 سنوات</t>
         </is>
       </c>
-      <c r="I25" s="24" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>6,500 - 8,500 ج.م</t>
         </is>
       </c>
-      <c r="J25" s="24" t="inlineStr">
+      <c r="J25" s="6" t="inlineStr">
         <is>
           <t>8,500 - 11,000 ج.م</t>
         </is>
       </c>
-      <c r="K25" s="24" t="inlineStr">
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>مناسب لفرص الـ Junior .NET Development</t>
         </is>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="20" t="n">
+      <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="21" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>يوسف محمد سعيد</t>
         </is>
       </c>
-      <c r="C26" s="22" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Youssef Mohamed Said</t>
         </is>
       </c>
-      <c r="D26" s="23" t="inlineStr">
-        <is>
-          <t>+20 106 845 5824</t>
-        </is>
-      </c>
-      <c r="E26" s="22" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>01068455824</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>yuossefmohamed592@gmail.com</t>
         </is>
       </c>
-      <c r="F26" s="24" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Backend .NET Developer</t>
         </is>
       </c>
-      <c r="G26" s="24" t="inlineStr">
-        <is>
-          <t>مبرمج كود (غير مستحب لخدمة العملاء)</t>
-        </is>
-      </c>
-      <c r="H26" s="25" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>مبرمج كود (High Turnover)</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>1 سنوات</t>
         </is>
       </c>
-      <c r="I26" s="24" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>8,000 - 11,000 ج.م</t>
         </is>
       </c>
-      <c r="J26" s="24" t="inlineStr">
+      <c r="J26" s="6" t="inlineStr">
         <is>
           <t>11,000 - 14,000 ج.م</t>
         </is>
       </c>
-      <c r="K26" s="24" t="inlineStr">
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>مناسب لوظائف Junior .NET Developer</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="20" t="n">
+      <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="21" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>عمرو أحمد</t>
         </is>
       </c>
-      <c r="C27" s="22" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Amr Ahmed</t>
         </is>
       </c>
-      <c r="D27" s="23" t="inlineStr">
-        <is>
-          <t>+20 106 789 1234</t>
-        </is>
-      </c>
-      <c r="E27" s="22" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>01069111355</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>amr.ahmed20001451@gmail.com</t>
         </is>
       </c>
-      <c r="F27" s="24" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Frontend Developer (React)</t>
         </is>
       </c>
-      <c r="G27" s="24" t="inlineStr">
-        <is>
-          <t>مبرمج كود (غير مستحب لخدمة العملاء)</t>
-        </is>
-      </c>
-      <c r="H27" s="25" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>مبرمج كود (High Turnover)</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>1.5 سنوات</t>
         </is>
       </c>
-      <c r="I27" s="24" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>7,000 - 9,500 ج.م</t>
         </is>
       </c>
-      <c r="J27" s="24" t="inlineStr">
+      <c r="J27" s="6" t="inlineStr">
         <is>
           <t>9,500 - 12,000 ج.م</t>
         </is>
       </c>
-      <c r="K27" s="24" t="inlineStr">
+      <c r="K27" s="6" t="inlineStr">
         <is>
           <t>مناسب لوظائف Frontend Web Developer</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="26" t="n">
+      <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="27" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>مالايشامي سيثورامان</t>
         </is>
       </c>
-      <c r="C28" s="28" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Malaichamy Sethuraman</t>
         </is>
       </c>
-      <c r="D28" s="29" t="inlineStr">
-        <is>
-          <t>+91 98401 23456</t>
-        </is>
-      </c>
-      <c r="E28" s="28" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>+91 9894417693</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>malai.hopes@gmail.com</t>
         </is>
       </c>
-      <c r="F28" s="30" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>Application Support Specialist (India)</t>
         </is>
       </c>
-      <c r="G28" s="30" t="inlineStr">
-        <is>
-          <t>مستبعد (غير مصري / مقيم بالخارج)</t>
-        </is>
-      </c>
-      <c r="H28" s="31" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>مستبعد (غير مصري)</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
         <is>
           <t>8 سنوات</t>
         </is>
       </c>
-      <c r="I28" s="30" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J28" s="30" t="inlineStr">
+      <c r="J28" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K28" s="30" t="inlineStr">
+      <c r="K28" s="6" t="inlineStr">
         <is>
           <t>مستبعد (Non-Egyptian)</t>
         </is>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="26" t="n">
+      <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="27" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>كلام علي</t>
         </is>
       </c>
-      <c r="C29" s="28" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Kalam Ali</t>
         </is>
       </c>
-      <c r="D29" s="29" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>+91 7522033696</t>
         </is>
       </c>
-      <c r="E29" s="28" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>kalamali0203@gmail.com</t>
         </is>
       </c>
-      <c r="F29" s="30" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Banking Application Support (India)</t>
         </is>
       </c>
-      <c r="G29" s="30" t="inlineStr">
-        <is>
-          <t>مستبعد (غير مصري / مقيم بالخارج)</t>
-        </is>
-      </c>
-      <c r="H29" s="31" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>مستبعد (غير مصري)</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>4 سنوات</t>
         </is>
       </c>
-      <c r="I29" s="30" t="inlineStr">
+      <c r="I29" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J29" s="30" t="inlineStr">
+      <c r="J29" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K29" s="30" t="inlineStr">
+      <c r="K29" s="6" t="inlineStr">
         <is>
           <t>مستبعد (Non-Egyptian)</t>
         </is>

</xml_diff>